<commit_message>
Modified according to the latest version of the protocol (discont e switch 12 e 24 + restarter)
</commit_message>
<xml_diff>
--- a/i_test/test_D6_Table_1/g_output/D6_Table_1_abira.xlsx
+++ b/i_test/test_D6_Table_1/g_output/D6_Table_1_abira.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S34"/>
+  <dimension ref="A1:S40"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -750,92 +750,92 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>211</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>202</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>225</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>217</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>224</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>228</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>171</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>181</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>156</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>188</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>174</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>185</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>167</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>165</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>162</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>152</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>158</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>146</t>
         </is>
       </c>
     </row>
@@ -854,92 +854,92 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>48.5 (42 - 57.25)</t>
+          <t>50 (39 - 59)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>47 (38 - 57.5)</t>
+          <t>48 (40 - 58.75)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>48 (41 - 60)</t>
+          <t>52 (43 - 61)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>51 (39.5 - 66)</t>
+          <t>51 (39 - 61)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>46.5 (38.75 - 57.25)</t>
+          <t>49 (41 - 61)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>57 (43 - 66)</t>
+          <t>49 (40 - 59)</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>53 (38 - 57)</t>
+          <t>49 (38 - 59)</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>48.5 (40.25 - 57)</t>
+          <t>49 (40 - 60)</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>53.5 (41 - 57)</t>
+          <t>49 (37 - 59)</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>55 (39.5 - 68)</t>
+          <t>51.5 (39 - 61)</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>50 (38.5 - 55.75)</t>
+          <t>51 (38 - 62)</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>52 (40 - 59)</t>
+          <t>49 (41 - 61)</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>52 (41 - 63)</t>
+          <t>51 (41.5 - 60)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>49 (38 - 61)</t>
+          <t>53 (42 - 63)</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>47.5 (42.5 - 60)</t>
+          <t>51.5 (41 - 62)</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>52.5 (42.75 - 61.5)</t>
+          <t>51 (39 - 61)</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>54.5 (40.25 - 61.75)</t>
+          <t>50.5 (42 - 60)</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>51.5 (35.25 - 58)</t>
+          <t>50 (40.25 - 60)</t>
         </is>
       </c>
     </row>
@@ -951,92 +951,92 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>24 (46,2%)</t>
+          <t>121 (57,3%)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>19 (40,4%)</t>
+          <t>103 (51,0%)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>26 (51,0%)</t>
+          <t>111 (49,3%)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>20 (36,4%)</t>
+          <t>108 (49,8%)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>19 (47,5%)</t>
+          <t>116 (51,8%)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>30 (52,6%)</t>
+          <t>119 (52,2%)</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>20 (54,1%)</t>
+          <t>82 (48,0%)</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>31 (53,4%)</t>
+          <t>73 (40,3%)</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>20 (45,5%)</t>
+          <t>77 (49,4%)</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>20 (51,3%)</t>
+          <t>94 (50,0%)</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>25 (65,8%)</t>
+          <t>78 (44,8%)</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>17 (51,5%)</t>
+          <t>101 (54,6%)</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>19 (46,3%)</t>
+          <t>84 (50,3%)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>28 (57,1%)</t>
+          <t>76 (46,1%)</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>15 (34,1%)</t>
+          <t>66 (40,7%)</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>31 (59,6%)</t>
+          <t>71 (46,7%)</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>25 (54,3%)</t>
+          <t>80 (50,6%)</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>24 (48,0%)</t>
+          <t>76 (52,1%)</t>
         </is>
       </c>
     </row>
@@ -1055,92 +1055,92 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>38 (73,1%)</t>
+          <t>143 (67,8%)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>26 (55,3%)</t>
+          <t>136 (67,3%)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>35 (68,6%)</t>
+          <t>162 (72,0%)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>36 (65,5%)</t>
+          <t>154 (71,0%)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>26 (65,0%)</t>
+          <t>149 (66,5%)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>41 (71,9%)</t>
+          <t>144 (63,2%)</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>22 (59,5%)</t>
+          <t>112 (65,5%)</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>47 (81,0%)</t>
+          <t>121 (66,9%)</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>28 (63,6%)</t>
+          <t>111 (71,2%)</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>26 (66,7%)</t>
+          <t>113 (60,1%)</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>22 (57,9%)</t>
+          <t>114 (65,5%)</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>19 (57,6%)</t>
+          <t>136 (73,5%)</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>29 (70,7%)</t>
+          <t>109 (65,3%)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>34 (69,4%)</t>
+          <t>117 (70,9%)</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>33 (75,0%)</t>
+          <t>110 (67,9%)</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>41 (78,8%)</t>
+          <t>107 (70,4%)</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>29 (63,0%)</t>
+          <t>116 (73,4%)</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>36 (72,0%)</t>
+          <t>103 (70,5%)</t>
         </is>
       </c>
     </row>
@@ -1152,92 +1152,92 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>8 (15,4%)</t>
+          <t>14 (6,6%)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>3 (6,4%)</t>
+          <t>17 (8,4%)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2 (3,9%)</t>
+          <t>15 (6,7%)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>4 (7,3%)</t>
+          <t>21 (9,7%)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>6 (15,0%)</t>
+          <t>19 (8,5%)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>6 (10,5%)</t>
+          <t>18 (7,9%)</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>4 (10,8%)</t>
+          <t>13 (7,6%)</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>4 (6,9%)</t>
+          <t>18 (9,9%)</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2 (4,5%)</t>
+          <t>16 (10,3%)</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>8 (20,5%)</t>
+          <t>16 (8,5%)</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>1 (2,6%)</t>
+          <t>14 (8,0%)</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>3 (9,1%)</t>
+          <t>15 (8,1%)</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>4 (9,8%)</t>
+          <t>13 (7,8%)</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>5 (10,2%)</t>
+          <t>12 (7,3%)</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>4 (9,1%)</t>
+          <t>15 (9,3%)</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>8 (15,4%)</t>
+          <t>18 (11,8%)</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>4 (8,7%)</t>
+          <t>11 (7,0%)</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>8 (16,0%)</t>
+          <t>14 (9,6%)</t>
         </is>
       </c>
     </row>
@@ -1249,92 +1249,92 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>20 (38,5%)</t>
+          <t>92 (43,6%)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>19 (40,4%)</t>
+          <t>68 (33,7%)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>24 (47,1%)</t>
+          <t>92 (40,9%)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>25 (45,5%)</t>
+          <t>92 (42,4%)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>14 (35,0%)</t>
+          <t>90 (40,2%)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>27 (47,4%)</t>
+          <t>94 (41,2%)</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>17 (45,9%)</t>
+          <t>73 (42,7%)</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>21 (36,2%)</t>
+          <t>60 (33,1%)</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>18 (40,9%)</t>
+          <t>67 (42,9%)</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>16 (41,0%)</t>
+          <t>72 (38,3%)</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>12 (31,6%)</t>
+          <t>71 (40,8%)</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>15 (45,5%)</t>
+          <t>74 (40,0%)</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>18 (43,9%)</t>
+          <t>80 (47,9%)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>19 (38,8%)</t>
+          <t>75 (45,5%)</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>15 (34,1%)</t>
+          <t>63 (38,9%)</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>19 (36,5%)</t>
+          <t>62 (40,8%)</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>18 (39,1%)</t>
+          <t>70 (44,3%)</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>28 (56,0%)</t>
+          <t>58 (39,7%)</t>
         </is>
       </c>
     </row>
@@ -1346,92 +1346,92 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>6 (11,5%)</t>
+          <t>36 (17,1%)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>5 (10,6%)</t>
+          <t>37 (18,3%)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>13 (25,5%)</t>
+          <t>29 (12,9%)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>8 (14,5%)</t>
+          <t>32 (14,7%)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>9 (22,5%)</t>
+          <t>29 (12,9%)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>10 (17,5%)</t>
+          <t>40 (17,5%)</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>4 (10,8%)</t>
+          <t>29 (17,0%)</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>7 (12,1%)</t>
+          <t>13 (7,2%)</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>5 (11,4%)</t>
+          <t>18 (11,5%)</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>5 (12,8%)</t>
+          <t>22 (11,7%)</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>9 (23,7%)</t>
+          <t>24 (13,8%)</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>4 (12,1%)</t>
+          <t>37 (20,0%)</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>7 (17,1%)</t>
+          <t>22 (13,2%)</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>9 (18,4%)</t>
+          <t>26 (15,8%)</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>6 (13,6%)</t>
+          <t>26 (16,0%)</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>8 (15,4%)</t>
+          <t>22 (14,5%)</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>3 (6,5%)</t>
+          <t>16 (10,1%)</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>12 (24,0%)</t>
+          <t>27 (18,5%)</t>
         </is>
       </c>
     </row>
@@ -1443,92 +1443,92 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>45 (86,5%)</t>
+          <t>178 (84,4%)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>36 (76,6%)</t>
+          <t>176 (87,1%)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>45 (88,2%)</t>
+          <t>185 (82,2%)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>45 (81,8%)</t>
+          <t>188 (86,6%)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>37 (92,5%)</t>
+          <t>192 (85,7%)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>48 (84,2%)</t>
+          <t>194 (85,1%)</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>30 (81,1%)</t>
+          <t>149 (87,1%)</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>45 (77,6%)</t>
+          <t>149 (82,3%)</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>38 (86,4%)</t>
+          <t>126 (80,8%)</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>34 (87,2%)</t>
+          <t>152 (80,9%)</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>34 (89,5%)</t>
+          <t>138 (79,3%)</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>29 (87,9%)</t>
+          <t>159 (85,9%)</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>36 (87,8%)</t>
+          <t>146 (87,4%)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>44 (89,8%)</t>
+          <t>148 (89,7%)</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>38 (86,4%)</t>
+          <t>135 (83,3%)</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>45 (86,5%)</t>
+          <t>133 (87,5%)</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>40 (87,0%)</t>
+          <t>128 (81,0%)</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>41 (82,0%)</t>
+          <t>117 (80,1%)</t>
         </is>
       </c>
     </row>
@@ -1540,92 +1540,92 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>39 (75,0%)</t>
+          <t>182 (86,3%)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>39 (83,0%)</t>
+          <t>169 (83,7%)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>44 (86,3%)</t>
+          <t>178 (79,1%)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>42 (76,4%)</t>
+          <t>182 (83,9%)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>32 (80,0%)</t>
+          <t>184 (82,1%)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>46 (80,7%)</t>
+          <t>196 (86,0%)</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>34 (91,9%)</t>
+          <t>150 (87,7%)</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>49 (84,5%)</t>
+          <t>158 (87,3%)</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>37 (84,1%)</t>
+          <t>133 (85,3%)</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>29 (74,4%)</t>
+          <t>168 (89,4%)</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>31 (81,6%)</t>
+          <t>150 (86,2%)</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>28 (84,8%)</t>
+          <t>148 (80,0%)</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>32 (78,0%)</t>
+          <t>135 (80,8%)</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>41 (83,7%)</t>
+          <t>141 (85,5%)</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>41 (93,2%)</t>
+          <t>141 (87,0%)</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>46 (88,5%)</t>
+          <t>129 (84,9%)</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>42 (91,3%)</t>
+          <t>134 (84,8%)</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>42 (84,0%)</t>
+          <t>124 (84,9%)</t>
         </is>
       </c>
     </row>
@@ -1637,92 +1637,92 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>27 (51,9%)</t>
+          <t>97 (46,0%)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>23 (48,9%)</t>
+          <t>105 (52,0%)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>27 (52,9%)</t>
+          <t>124 (55,1%)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>32 (58,2%)</t>
+          <t>107 (49,3%)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>20 (50,0%)</t>
+          <t>114 (50,9%)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>25 (43,9%)</t>
+          <t>128 (56,1%)</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>16 (43,2%)</t>
+          <t>88 (51,5%)</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>27 (46,6%)</t>
+          <t>102 (56,4%)</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>16 (36,4%)</t>
+          <t>80 (51,3%)</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>24 (61,5%)</t>
+          <t>106 (56,4%)</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>21 (55,3%)</t>
+          <t>94 (54,0%)</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>11 (33,3%)</t>
+          <t>109 (58,9%)</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>25 (61,0%)</t>
+          <t>81 (48,5%)</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>29 (59,2%)</t>
+          <t>79 (47,9%)</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>27 (61,4%)</t>
+          <t>85 (52,5%)</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>36 (69,2%)</t>
+          <t>87 (57,2%)</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>25 (54,3%)</t>
+          <t>86 (54,4%)</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>24 (48,0%)</t>
+          <t>71 (48,6%)</t>
         </is>
       </c>
     </row>
@@ -1734,92 +1734,92 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>6 (11,5%)</t>
+          <t>44 (20,9%)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>10 (21,3%)</t>
+          <t>46 (22,8%)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>14 (27,5%)</t>
+          <t>52 (23,1%)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>13 (23,6%)</t>
+          <t>39 (18,0%)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>9 (22,5%)</t>
+          <t>55 (24,6%)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>14 (24,6%)</t>
+          <t>39 (17,1%)</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>10 (27,0%)</t>
+          <t>34 (19,9%)</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>5 (8,6%)</t>
+          <t>33 (18,2%)</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>7 (15,9%)</t>
+          <t>24 (15,4%)</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>10 (25,6%)</t>
+          <t>29 (15,4%)</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>7 (18,4%)</t>
+          <t>28 (16,1%)</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>3 (9,1%)</t>
+          <t>34 (18,4%)</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>10 (24,4%)</t>
+          <t>23 (13,8%)</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>9 (18,4%)</t>
+          <t>28 (17,0%)</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>5 (11,4%)</t>
+          <t>33 (20,4%)</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>5 (9,6%)</t>
+          <t>22 (14,5%)</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>13 (28,3%)</t>
+          <t>27 (17,1%)</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>11 (22,0%)</t>
+          <t>33 (22,6%)</t>
         </is>
       </c>
     </row>
@@ -1831,92 +1831,92 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>5 (9,6%)</t>
+          <t>18 (8,5%)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>5 (10,6%)</t>
+          <t>17 (8,4%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>4 (7,8%)</t>
+          <t>20 (8,9%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>0 (0,0%)</t>
+          <t>22 (10,1%)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>3 (7,5%)</t>
+          <t>22 (9,8%)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2 (3,5%)</t>
+          <t>16 (7,0%)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>3 (8,1%)</t>
+          <t>17 (9,9%)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>4 (6,9%)</t>
+          <t>16 (8,8%)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>5 (11,4%)</t>
+          <t>9 (5,8%)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>1 (2,6%)</t>
+          <t>24 (12,8%)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>4 (10,5%)</t>
+          <t>18 (10,3%)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>5 (15,2%)</t>
+          <t>15 (8,1%)</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>3 (7,3%)</t>
+          <t>10 (6,0%)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>5 (10,2%)</t>
+          <t>15 (9,1%)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>6 (13,6%)</t>
+          <t>13 (8,0%)</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>2 (3,8%)</t>
+          <t>11 (7,2%)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>4 (8,7%)</t>
+          <t>8 (5,1%)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>7 (14,0%)</t>
+          <t>7 (4,8%)</t>
         </is>
       </c>
     </row>
@@ -1928,92 +1928,92 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>47 (90,4%)</t>
+          <t>190 (90,0%)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>42 (89,4%)</t>
+          <t>181 (89,6%)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>48 (94,1%)</t>
+          <t>200 (88,9%)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>48 (87,3%)</t>
+          <t>188 (86,6%)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>33 (82,5%)</t>
+          <t>196 (87,5%)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>49 (86,0%)</t>
+          <t>197 (86,4%)</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>33 (89,2%)</t>
+          <t>152 (88,9%)</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>48 (82,8%)</t>
+          <t>163 (90,1%)</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>41 (93,2%)</t>
+          <t>141 (90,4%)</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>33 (84,6%)</t>
+          <t>161 (85,6%)</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>31 (81,6%)</t>
+          <t>148 (85,1%)</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>24 (72,7%)</t>
+          <t>155 (83,8%)</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>34 (82,9%)</t>
+          <t>150 (89,8%)</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>45 (91,8%)</t>
+          <t>145 (87,9%)</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>41 (93,2%)</t>
+          <t>140 (86,4%)</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>44 (84,6%)</t>
+          <t>128 (84,2%)</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>39 (84,8%)</t>
+          <t>143 (90,5%)</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>44 (88,0%)</t>
+          <t>127 (87,0%)</t>
         </is>
       </c>
     </row>
@@ -2025,92 +2025,92 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>48 (92,3%)</t>
+          <t>200 (94,8%)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>46 (97,9%)</t>
+          <t>191 (94,6%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>48 (94,1%)</t>
+          <t>213 (94,7%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>52 (94,5%)</t>
+          <t>209 (96,3%)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>35 (87,5%)</t>
+          <t>213 (95,1%)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>55 (96,5%)</t>
+          <t>209 (91,7%)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>32 (86,5%)</t>
+          <t>156 (91,2%)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>53 (91,4%)</t>
+          <t>172 (95,0%)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>42 (95,5%)</t>
+          <t>146 (93,6%)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>35 (89,7%)</t>
+          <t>180 (95,7%)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>37 (97,4%)</t>
+          <t>164 (94,3%)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>32 (97,0%)</t>
+          <t>177 (95,7%)</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>38 (92,7%)</t>
+          <t>155 (92,8%)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>40 (81,6%)</t>
+          <t>150 (90,9%)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>41 (93,2%)</t>
+          <t>153 (94,4%)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>48 (92,3%)</t>
+          <t>141 (92,8%)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>42 (91,3%)</t>
+          <t>147 (93,0%)</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>45 (90,0%)</t>
+          <t>138 (94,5%)</t>
         </is>
       </c>
     </row>
@@ -2122,92 +2122,92 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>5 (3 - 7)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
           <t>4 (2 - 6)</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>4 (3 - 7)</t>
-        </is>
-      </c>
       <c r="D21" t="inlineStr">
         <is>
+          <t>4 (2 - 6)</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>4 (3 - 6)</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>4 (2 - 6)</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>4 (2.75 - 6)</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>4 (3 - 6)</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>4 (3 - 6)</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>4 (3 - 6)</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>4.5 (2 - 6)</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>5 (3 - 6)</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>4 (2 - 6)</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>4 (3 - 6)</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
           <t>5 (3 - 7)</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>5 (3 - 6)</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>4 (3 - 7)</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>5 (3 - 7)</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>4 (2 - 7)</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>4.5 (2.25 - 6)</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>4 (3 - 6.25)</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
+      <c r="P21" t="inlineStr">
         <is>
           <t>4 (3 - 6)</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>4.5 (2.25 - 6)</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>4 (3 - 6)</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>5 (2 - 6)</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
         <is>
           <t>4 (2 - 6)</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>4 (2 - 6)</t>
-        </is>
-      </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>4 (3 - 6)</t>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>4 (2 - 5.25)</t>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>4 (2 - 6.75)</t>
-        </is>
-      </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>5 (3 - 6)</t>
+          <t>4.5 (3 - 7)</t>
         </is>
       </c>
     </row>
@@ -2226,92 +2226,92 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>31 (59,6%)</t>
+          <t>132 (62,6%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>29 (61,7%)</t>
+          <t>121 (59,9%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>32 (62,7%)</t>
+          <t>138 (61,3%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>30 (54,5%)</t>
+          <t>131 (60,4%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>23 (57,5%)</t>
+          <t>135 (60,3%)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>39 (68,4%)</t>
+          <t>144 (63,2%)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>24 (64,9%)</t>
+          <t>103 (60,2%)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>34 (58,6%)</t>
+          <t>113 (62,4%)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>31 (70,5%)</t>
+          <t>104 (66,7%)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>26 (66,7%)</t>
+          <t>126 (67,0%)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>23 (60,5%)</t>
+          <t>114 (65,5%)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>22 (66,7%)</t>
+          <t>113 (61,1%)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>24 (58,5%)</t>
+          <t>109 (65,3%)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>32 (65,3%)</t>
+          <t>105 (63,6%)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>28 (63,6%)</t>
+          <t>100 (61,7%)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>31 (59,6%)</t>
+          <t>89 (58,6%)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>33 (71,7%)</t>
+          <t>87 (55,1%)</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>33 (66,0%)</t>
+          <t>85 (58,2%)</t>
         </is>
       </c>
     </row>
@@ -2323,92 +2323,92 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>38 (73,1%)</t>
+          <t>153 (72,5%)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>36 (76,6%)</t>
+          <t>130 (64,4%)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>28 (54,9%)</t>
+          <t>150 (66,7%)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>37 (67,3%)</t>
+          <t>163 (75,1%)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>24 (60,0%)</t>
+          <t>141 (62,9%)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>35 (61,4%)</t>
+          <t>150 (65,8%)</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>25 (67,6%)</t>
+          <t>108 (63,2%)</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>40 (69,0%)</t>
+          <t>124 (68,5%)</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>27 (61,4%)</t>
+          <t>106 (67,9%)</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>31 (79,5%)</t>
+          <t>117 (62,2%)</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>24 (63,2%)</t>
+          <t>114 (65,5%)</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>12 (36,4%)</t>
+          <t>110 (59,5%)</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>27 (65,9%)</t>
+          <t>107 (64,1%)</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>37 (75,5%)</t>
+          <t>111 (67,3%)</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>28 (63,6%)</t>
+          <t>108 (66,7%)</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>36 (69,2%)</t>
+          <t>97 (63,8%)</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>32 (69,6%)</t>
+          <t>104 (65,8%)</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>34 (68,0%)</t>
+          <t>105 (71,9%)</t>
         </is>
       </c>
     </row>
@@ -2420,92 +2420,92 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>16 (30,8%)</t>
+          <t>75 (35,5%)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>12 (25,5%)</t>
+          <t>69 (34,2%)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>16 (31,4%)</t>
+          <t>65 (28,9%)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>14 (25,5%)</t>
+          <t>80 (36,9%)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>16 (40,0%)</t>
+          <t>79 (35,3%)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>18 (31,6%)</t>
+          <t>90 (39,5%)</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>15 (40,5%)</t>
+          <t>56 (32,7%)</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>20 (34,5%)</t>
+          <t>57 (31,5%)</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>14 (31,8%)</t>
+          <t>56 (35,9%)</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>10 (25,6%)</t>
+          <t>55 (29,3%)</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>11 (28,9%)</t>
+          <t>62 (35,6%)</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>13 (39,4%)</t>
+          <t>59 (31,9%)</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>13 (31,7%)</t>
+          <t>54 (32,3%)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>20 (40,8%)</t>
+          <t>58 (35,2%)</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>16 (36,4%)</t>
+          <t>53 (32,7%)</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>13 (25,0%)</t>
+          <t>43 (28,3%)</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>17 (37,0%)</t>
+          <t>54 (34,2%)</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>14 (28,0%)</t>
+          <t>58 (39,7%)</t>
         </is>
       </c>
     </row>
@@ -2517,92 +2517,92 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>20 (38,5%)</t>
+          <t>86 (40,8%)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>16 (34,0%)</t>
+          <t>80 (39,6%)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>19 (37,3%)</t>
+          <t>76 (33,8%)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>15 (27,3%)</t>
+          <t>77 (35,5%)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>19 (47,5%)</t>
+          <t>81 (36,2%)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>21 (36,8%)</t>
+          <t>88 (38,6%)</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>12 (32,4%)</t>
+          <t>69 (40,4%)</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>21 (36,2%)</t>
+          <t>63 (34,8%)</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>15 (34,1%)</t>
+          <t>54 (34,6%)</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>16 (41,0%)</t>
+          <t>67 (35,6%)</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>17 (44,7%)</t>
+          <t>63 (36,2%)</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>16 (48,5%)</t>
+          <t>75 (40,5%)</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>10 (24,4%)</t>
+          <t>49 (29,3%)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>20 (40,8%)</t>
+          <t>64 (38,8%)</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>14 (31,8%)</t>
+          <t>56 (34,6%)</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>19 (36,5%)</t>
+          <t>61 (40,1%)</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>15 (32,6%)</t>
+          <t>55 (34,8%)</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>22 (44,0%)</t>
+          <t>44 (30,1%)</t>
         </is>
       </c>
     </row>
@@ -2614,92 +2614,92 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>7 (13,5%)</t>
+          <t>15 (7,1%)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>4 (8,5%)</t>
+          <t>20 (9,9%)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>5 (9,8%)</t>
+          <t>19 (8,4%)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>6 (10,9%)</t>
+          <t>20 (9,2%)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2 (5,0%)</t>
+          <t>14 (6,2%)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>5 (8,8%)</t>
+          <t>15 (6,6%)</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>3 (8,1%)</t>
+          <t>10 (5,8%)</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>4 (6,9%)</t>
+          <t>17 (9,4%)</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2 (4,5%)</t>
+          <t>10 (6,4%)</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>3 (7,7%)</t>
+          <t>15 (8,0%)</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>4 (10,5%)</t>
+          <t>13 (7,5%)</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>3 (9,1%)</t>
+          <t>13 (7,0%)</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>4 (9,8%)</t>
+          <t>13 (7,8%)</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>2 (4,1%)</t>
+          <t>13 (7,9%)</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>2 (4,5%)</t>
+          <t>14 (8,6%)</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>4 (7,7%)</t>
+          <t>9 (5,9%)</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>4 (8,7%)</t>
+          <t>16 (10,1%)</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>5 (10,0%)</t>
+          <t>9 (6,2%)</t>
         </is>
       </c>
     </row>
@@ -2711,494 +2711,1166 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>15 (28,8%)</t>
+          <t>80 (37,9%)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>16 (34,0%)</t>
+          <t>73 (36,1%)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>20 (39,2%)</t>
+          <t>87 (38,7%)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>21 (38,2%)</t>
+          <t>75 (34,6%)</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>15 (37,5%)</t>
+          <t>88 (39,3%)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>20 (35,1%)</t>
+          <t>98 (43,0%)</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>11 (29,7%)</t>
+          <t>71 (41,5%)</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>21 (36,2%)</t>
+          <t>55 (30,4%)</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>18 (40,9%)</t>
+          <t>59 (37,8%)</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>20 (51,3%)</t>
+          <t>69 (36,7%)</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>8 (21,1%)</t>
+          <t>56 (32,2%)</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>14 (42,4%)</t>
+          <t>69 (37,3%)</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>10 (24,4%)</t>
+          <t>73 (43,7%)</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>17 (34,7%)</t>
+          <t>62 (37,6%)</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>15 (34,1%)</t>
+          <t>66 (40,7%)</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>17 (32,7%)</t>
+          <t>55 (36,2%)</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>15 (32,6%)</t>
+          <t>61 (38,6%)</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>14 (28,0%)</t>
+          <t>48 (32,9%)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Interruzione trattamento</t>
+          <t>Interruzione trattamento a 12 mesi</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>203 (96,2%)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>193 (95,5%)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>219 (97,3%)</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>211 (97,2%)</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>214 (95,5%)</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>220 (96,5%)</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>167 (97,7%)</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>179 (98,9%)</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>154 (98,7%)</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>186 (98,9%)</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>170 (97,7%)</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>181 (97,8%)</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>163 (97,6%)</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>160 (97,0%)</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>157 (96,9%)</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>148 (97,4%)</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>152 (96,2%)</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>139 (95,2%)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Switch</t>
+          <t>Interruzione trattamento a 24 mesi</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>163 (77,3%)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>147 (72,8%)</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>168 (74,7%)</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>152 (70,0%)</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>163 (72,8%)</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>170 (74,6%)</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>132 (77,2%)</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>130 (71,8%)</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>111 (71,2%)</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>141 (75,0%)</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>125 (71,8%)</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>129 (69,7%)</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>129 (77,2%)</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>114 (69,1%)</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>115 (71,0%)</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>106 (69,7%)</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>110 (69,6%)</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>116 (79,5%)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Vs apalutamide</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>6 (11,5%)</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>4 (8,5%)</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>9 (17,6%)</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>9 (16,4%)</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>8 (20,0%)</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>7 (12,3%)</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>1 (2,7%)</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>5 (8,6%)</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>3 (6,8%)</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>8 (20,5%)</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>8 (21,1%)</t>
-        </is>
-      </c>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>5 (15,2%)</t>
-        </is>
-      </c>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>2 (4,9%)</t>
-        </is>
-      </c>
-      <c r="O31" t="inlineStr">
-        <is>
-          <t>6 (12,2%)</t>
-        </is>
-      </c>
-      <c r="P31" t="inlineStr">
-        <is>
-          <t>3 (6,8%)</t>
-        </is>
-      </c>
-      <c r="Q31" t="inlineStr">
-        <is>
-          <t>2 (3,8%)</t>
-        </is>
-      </c>
-      <c r="R31" t="inlineStr">
-        <is>
-          <t>8 (17,4%)</t>
-        </is>
-      </c>
-      <c r="S31" t="inlineStr">
-        <is>
-          <t>6 (12,0%)</t>
+          <t>Switch</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Vs enzalutamide</t>
+          <t>Vs apalutamide a 12 mesi</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>7 (13,5%)</t>
+          <t>26 (12,3%)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>4 (8,5%)</t>
+          <t>20 (9,9%)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2 (3,9%)</t>
+          <t>25 (11,1%)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2 (3,6%)</t>
+          <t>27 (12,4%)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>3 (7,5%)</t>
+          <t>27 (12,1%)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>6 (10,5%)</t>
+          <t>28 (12,3%)</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>1 (2,7%)</t>
+          <t>24 (14,0%)</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>6 (10,3%)</t>
+          <t>18 (9,9%)</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>3 (6,8%)</t>
+          <t>20 (12,8%)</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2 (5,1%)</t>
+          <t>23 (12,2%)</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>7 (18,4%)</t>
+          <t>13 (7,5%)</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>1 (3,0%)</t>
+          <t>27 (14,6%)</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2 (4,9%)</t>
+          <t>19 (11,4%)</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>7 (14,3%)</t>
+          <t>18 (10,9%)</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>3 (6,8%)</t>
+          <t>18 (11,1%)</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>6 (11,5%)</t>
+          <t>17 (11,2%)</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>5 (10,9%)</t>
+          <t>23 (14,6%)</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>12 (24,0%)</t>
+          <t>20 (13,7%)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Vs darolutamide</t>
+          <t>Vs enzalutamide a 12 mesi</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>41 (78,8%)</t>
+          <t>22 (10,4%)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>36 (76,6%)</t>
+          <t>25 (12,4%)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>43 (84,3%)</t>
+          <t>25 (11,1%)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>49 (89,1%)</t>
+          <t>11 (5,1%)</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>35 (87,5%)</t>
+          <t>21 (9,4%)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>47 (82,5%)</t>
+          <t>20 (8,8%)</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>30 (81,1%)</t>
+          <t>14 (8,2%)</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>49 (84,5%)</t>
+          <t>16 (8,8%)</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>34 (77,3%)</t>
+          <t>9 (5,8%)</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>33 (84,6%)</t>
+          <t>17 (9,0%)</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>33 (86,8%)</t>
+          <t>19 (10,9%)</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>29 (87,9%)</t>
+          <t>23 (12,4%)</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>34 (82,9%)</t>
+          <t>17 (10,2%)</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>41 (83,7%)</t>
+          <t>17 (10,3%)</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>33 (75,0%)</t>
+          <t>10 (6,2%)</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>43 (82,7%)</t>
+          <t>17 (11,2%)</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>43 (93,5%)</t>
+          <t>19 (12,0%)</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>46 (92,0%)</t>
+          <t>19 (13,0%)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Vs altri farmaci oncologici (L01)</t>
+          <t>Vs darolutamide a 12 mesi</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>18 (34,6%)</t>
+          <t>170 (80,6%)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>14 (29,8%)</t>
+          <t>168 (83,2%)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>25 (49,0%)</t>
+          <t>180 (80,0%)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>16 (29,1%)</t>
+          <t>172 (79,3%)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>12 (30,0%)</t>
+          <t>178 (79,5%)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>25 (43,9%)</t>
+          <t>191 (83,8%)</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>12 (32,4%)</t>
+          <t>139 (81,3%)</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>24 (41,4%)</t>
+          <t>144 (79,6%)</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>15 (34,1%)</t>
+          <t>131 (84,0%)</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>13 (33,3%)</t>
+          <t>140 (74,5%)</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>14 (36,8%)</t>
+          <t>141 (81,0%)</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>14 (42,4%)</t>
+          <t>140 (75,7%)</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>9 (22,0%)</t>
+          <t>136 (81,4%)</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>15 (30,6%)</t>
+          <t>137 (83,0%)</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>17 (38,6%)</t>
+          <t>135 (83,3%)</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>18 (34,6%)</t>
+          <t>127 (83,6%)</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>17 (37,0%)</t>
+          <t>138 (87,3%)</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>16 (32,0%)</t>
+          <t>124 (84,9%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Vs altri farmaci oncologici (L01) a 12 mesi</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>59 (28,0%)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>71 (35,1%)</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>71 (31,6%)</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>69 (31,8%)</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>79 (35,3%)</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>77 (33,8%)</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>47 (27,5%)</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>60 (33,1%)</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>54 (34,6%)</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>71 (37,8%)</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>50 (28,7%)</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>67 (36,2%)</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>56 (33,5%)</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>48 (29,1%)</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>51 (31,5%)</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>48 (31,6%)</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>45 (28,5%)</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>40 (27,4%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Vs apalutamide a 24 mesi</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>148 (70,1%)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>143 (70,8%)</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>159 (70,7%)</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>151 (69,6%)</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>153 (68,3%)</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>142 (62,3%)</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>122 (71,3%)</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>128 (70,7%)</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>119 (76,3%)</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>122 (64,9%)</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>125 (71,8%)</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>130 (70,3%)</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>115 (68,9%)</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>117 (70,9%)</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>102 (63,0%)</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>106 (69,7%)</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>114 (72,2%)</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>103 (70,5%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Vs enzalutamide a 24 mesi</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>36 (17,1%)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>30 (14,9%)</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>35 (15,6%)</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>21 (9,7%)</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>30 (13,4%)</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>30 (13,2%)</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>27 (15,8%)</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>27 (14,9%)</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>21 (13,5%)</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>28 (14,9%)</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>29 (16,7%)</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>37 (20,0%)</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>32 (19,2%)</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>27 (16,4%)</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>25 (15,4%)</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>27 (17,8%)</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>23 (14,6%)</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>17 (11,6%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Vs darolutamide a 24 mesi</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>195 (92,4%)</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>179 (88,6%)</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>201 (89,3%)</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>204 (94,0%)</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>199 (88,8%)</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>205 (89,9%)</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>153 (89,5%)</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>166 (91,7%)</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>140 (89,7%)</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>173 (92,0%)</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>153 (87,9%)</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>167 (90,3%)</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>151 (90,4%)</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>148 (89,7%)</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>149 (92,0%)</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>140 (92,1%)</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>139 (88,0%)</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>131 (89,7%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Vs altri farmaci oncologici (L01) a 24 mesi</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>25 (11,8%)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>22 (10,9%)</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>30 (13,3%)</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>32 (14,7%)</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>26 (11,6%)</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>19 (8,3%)</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>25 (14,6%)</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>17 (9,4%)</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>26 (16,7%)</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>25 (13,3%)</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>20 (11,5%)</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>17 (9,2%)</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>23 (13,8%)</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>18 (10,9%)</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>15 (9,3%)</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>15 (9,9%)</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>14 (8,9%)</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>15 (10,3%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Ri-iniziatori</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>141 (66,8%)</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>136 (67,3%)</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>146 (64,9%)</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>129 (59,4%)</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>138 (61,6%)</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>144 (63,2%)</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>100 (58,5%)</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>107 (59,1%)</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>94 (60,3%)</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>120 (63,8%)</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>114 (65,5%)</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>124 (67,0%)</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>107 (64,1%)</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>101 (61,2%)</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>104 (64,2%)</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>91 (59,9%)</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>113 (71,5%)</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>93 (63,7%)</t>
         </is>
       </c>
     </row>

</xml_diff>